<commit_message>
Add GitHub Actions workflows
</commit_message>
<xml_diff>
--- a/data/airline_data.xlsx
+++ b/data/airline_data.xlsx
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>1</v>
@@ -571,7 +571,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Иван Пассажир</t>
+          <t>Иван Пасспавв</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -712,7 +712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -798,7 +798,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SM-101</t>
+          <t>SM-102</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -835,22 +835,22 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K2" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="L2" t="n">
-        <v>12500</v>
+        <v>12503</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Задерживается</t>
+          <t>Отменен</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Flexible</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -865,50 +865,50 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SM-202</t>
+          <t>нпрпеар</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Санкт-Петербург</t>
+          <t>рапрапр</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Казань</t>
+          <t>рапра</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-04</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>13:05</t>
         </is>
       </c>
       <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Airbus A320</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
         <v>3</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Sukhoi Superjet 100</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>98</v>
-      </c>
       <c r="K3" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
-        <v>7900</v>
+        <v>4234234</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -917,146 +917,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Flexible</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-04-08 23:27:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SM-303</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Екатеринбург</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Новосибирск</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>07:45</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>10:20</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Boeing 737-800</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>189</v>
-      </c>
-      <c r="K4" t="n">
-        <v>121</v>
-      </c>
-      <c r="L4" t="n">
-        <v>9800</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Задерживается</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Promo</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>2026-04-08 23:27:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SM-404</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Москва</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Калининград</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>20:15</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>3</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Sukhoi Superjet 100</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>98</v>
-      </c>
-      <c r="K5" t="n">
-        <v>47</v>
-      </c>
-      <c r="L5" t="n">
-        <v>8900</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>По расписанию</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>2026-04-08 23:27:55</t>
+          <t>2026-04-29 23:10:02</t>
         </is>
       </c>
     </row>
@@ -1071,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1188,6 +1054,216 @@
         </is>
       </c>
       <c r="L2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BK-100002</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SM-101</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>екупупу</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>50</v>
+      </c>
+      <c r="I3" t="n">
+        <v>6250</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>cancelled</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:03:36</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:03:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BK-100003</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SM-101</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>купупуепу</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>loyal</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I4" t="n">
+        <v>10625</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>cancelled</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:03:36</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:07:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BK-100004</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SM-102</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>пкпвап</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>12503</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:08:05</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BK-100005</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SM-102</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>пвапавпв</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>50</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6251</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:08:05</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1293,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1388,6 +1464,576 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:02:25</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Вход client@skymanager.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:02:48</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Профиль обновлен</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:02:57</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Профиль обновлен</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:03:36</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>booking</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Оформлено мест: 2 на рейс SM-101</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:03:45</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>cancel_booking</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Отменено бронирование BK-100002</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:04:28</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>employee@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>employee</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Вход employee@skymanager.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:05:05</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>employee@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>employee</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>save_flight</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Сохранен рейс SM-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:07:23</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Вход client@skymanager.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:07:28</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>cancel_booking</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Отменено бронирование BK-100003</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:07:39</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Профиль обновлен</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:07:45</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Профиль обновлен</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:07:49</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Профиль обновлен</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:08:05</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>client@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>booking</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Оформлено мест: 2 на рейс SM-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:08:31</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>admin@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>login</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Вход admin@skymanager.local</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:09:38</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>admin@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>save_flight</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Сохранен рейс SM-102</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:09:40</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>admin@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>delete_flight</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Удален рейс 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:09:42</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>admin@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>delete_flight</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Удален рейс 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:09:43</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>admin@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>delete_flight</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Удален рейс 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-04-29 23:10:02</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>admin@skymanager.local</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>save_flight</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Сохранен рейс нпрпеар</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>